<commit_message>
feat(analytics): add fair probabilities, sharp reversal detection and enriched drift reporting
</commit_message>
<xml_diff>
--- a/data/reports/dq_report_latest.xlsx
+++ b/data/reports/dq_report_latest.xlsx
@@ -2282,7 +2282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2294,6 +2294,12 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2342,6 +2348,36 @@
           <t>Date snapshot actuel</t>
         </is>
       </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Ancienne proba (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Nouvelle proba (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Gain de proba (pts)</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Cote Fair actuelle</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Signal Marché</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Reversal Intensity (%)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(engine): add odds-drift tracking, clv analysis, dynamic seeds and robust date parsing
</commit_message>
<xml_diff>
--- a/data/reports/dq_report_latest.xlsx
+++ b/data/reports/dq_report_latest.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Synthèse DQ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Clean Odds" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="DQ Exceptions Log" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Market Trends &amp; Drift" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CLV Backtest Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Analyse Odds Drift" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="166" formatCode="0.00&quot;%&quot;"/>
+    <numFmt numFmtId="167" formatCode="+0.00%;-0.00%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -98,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -118,15 +121,49 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FCE8E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="007030A0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E4DFEC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -502,7 +539,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Executive Summary</t>
+          <t>Synthèse DQ</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -530,7 +567,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5">
@@ -540,7 +577,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -560,12 +597,18 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0.4</v>
+        <v>0.4827586206896552</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Taux de battement CLV (%)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.125</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -611,12 +654,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -674,16 +717,16 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>46305.47916666666</v>
+        <v>46292.54166666666</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>AEL Larissa</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>PAOK B</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -692,33 +735,33 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.38</v>
+        <v>1.33</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4.83</v>
+        <v>4.19</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>7.74</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>106.0876</v>
+        <v>110.88864</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>46305.58333333334</v>
+        <v>46292.54166666666</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Kalamaria</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Karditsa</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -727,33 +770,33 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2.59</v>
+        <v>3.32</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>3.53</v>
+        <v>2.93</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2.55</v>
+        <v>2.14</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>106.15434</v>
+        <v>110.97915</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>46305.58333333334</v>
+        <v>46292.54166666666</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Niki Volos</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Chrisoupolis</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -762,33 +805,33 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1.79</v>
+        <v>1.22</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>4.02</v>
+        <v>4.38</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>3.94</v>
+        <v>15.17</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>106.12225</v>
+        <v>111.39022</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46305.58333333334</v>
+        <v>46292.54166666666</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Panionios</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Zakynthos</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -797,33 +840,33 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2.68</v>
+        <v>1.21</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3.47</v>
+        <v>4.73</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>2.49</v>
+        <v>13.63</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>106.29252</v>
+        <v>111.12303</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>46305.58333333334</v>
+        <v>46292.58333333334</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Ellas Syrou</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Pyrgos</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -832,33 +875,33 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2.9</v>
+        <v>1.65</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>3.45</v>
+        <v>3.44</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2.34</v>
+        <v>4.82</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>106.20331</v>
+        <v>110.42272</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46305.6875</v>
+        <v>46292.63541666666</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Man United</t>
+          <t>Panserraikos</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>Olympiacos Piraeus B</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -867,33 +910,33 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1.71</v>
+        <v>1.27</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>4.1</v>
+        <v>4.42</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>4.32</v>
+        <v>11</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>106.01792</v>
+        <v>110.4555</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>46306.54166666666</v>
+        <v>46293.54166666666</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace</t>
+          <t>Athens Kallithea</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nott'm Forest</t>
+          <t>Asteras Tripolis B</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -902,33 +945,33 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>3.32</v>
+        <v>3.35</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>2.66</v>
+        <v>5.38</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>106.17601</v>
+        <v>110.93811</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46306.54166666666</v>
+        <v>46293.54166666666</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Marko</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>Panthrakikos</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -937,33 +980,33 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3.6</v>
+        <v>1.41</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>3.35</v>
+        <v>3.9</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>2.06</v>
+        <v>6.77</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>106.17221</v>
+        <v>111.33406</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>46291.39188657407</v>
+        <v>46291.49375</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>46306.64583333334</v>
+        <v>46305.47916666666</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Man City</t>
+          <t>Leeds</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -972,16 +1015,16 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2.58</v>
+        <v>1.38</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>3.66</v>
+        <v>4.83</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2.49</v>
+        <v>7.74</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>106.24274</v>
+        <v>106.0876</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>46291.39188657407</v>
@@ -989,16 +1032,16 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46307.79166666666</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Newcastle</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1007,16 +1050,16 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.28</v>
+        <v>2.59</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>3.61</v>
+        <v>3.53</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>2.09</v>
+        <v>2.55</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>106.03553</v>
+        <v>106.15434</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1024,16 +1067,16 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>46312.47916666666</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1042,16 +1085,16 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>2.84</v>
+        <v>1.79</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>3.68</v>
+        <v>4.02</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>2.26</v>
+        <v>3.94</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>106.63297</v>
+        <v>106.12225</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1059,16 +1102,16 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>46312.58333333334</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1077,16 +1120,16 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2.71</v>
+        <v>2.68</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>3.64</v>
+        <v>3.47</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>2.37</v>
+        <v>2.49</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>106.56699</v>
+        <v>106.29252</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1094,16 +1137,16 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>46312.58333333334</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Brighton</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1112,16 +1155,16 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1.66</v>
+        <v>2.9</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>3.99</v>
+        <v>3.45</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>4.77</v>
+        <v>2.34</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>106.26798</v>
+        <v>106.20331</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1129,16 +1172,16 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>46312.58333333334</v>
+        <v>46305.6875</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Man City</t>
+          <t>Man United</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Tottenham</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1147,16 +1190,16 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1.22</v>
+        <v>1.71</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>6.57</v>
+        <v>4.1</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>10.67</v>
+        <v>4.32</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>106.55998</v>
+        <v>106.01792</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1164,16 +1207,16 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>46312.6875</v>
+        <v>46306.54166666666</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Newcastle</t>
+          <t>Crystal Palace</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Nott'm Forest</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1182,16 +1225,16 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2.07</v>
+        <v>2.6</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>3.72</v>
+        <v>3.32</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>3.19</v>
+        <v>2.66</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>106.53886</v>
+        <v>106.17601</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1199,16 +1242,16 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>46313.54166666666</v>
+        <v>46306.54166666666</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1217,16 +1260,16 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1.99</v>
+        <v>3.6</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>3.56</v>
+        <v>3.35</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>3.56</v>
+        <v>2.06</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>106.43103</v>
+        <v>106.17221</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1234,16 +1277,16 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>46313.54166666666</v>
+        <v>46306.64583333334</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Crystal Palace</t>
+          <t>Man City</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1252,16 +1295,16 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>1.54</v>
+        <v>2.58</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>4.39</v>
+        <v>3.66</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>5.32</v>
+        <v>2.49</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>106.5111</v>
+        <v>106.24274</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1269,16 +1312,16 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>46313.54166666666</v>
+        <v>46307.79166666666</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Coventry</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Man United</t>
+          <t>Newcastle</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1287,16 +1330,16 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2.83</v>
+        <v>3.28</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>3.56</v>
+        <v>3.61</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2.33</v>
+        <v>2.09</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>106.34403</v>
+        <v>106.03553</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1304,16 +1347,16 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>46313.64583333334</v>
+        <v>46312.47916666666</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Nott'm Forest</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1322,16 +1365,16 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>5.58</v>
+        <v>2.84</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>3.88</v>
+        <v>3.68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1.59</v>
+        <v>2.26</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>106.58742</v>
+        <v>106.63297</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>46291.39188657407</v>
@@ -1339,36 +1382,316 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>106.56699</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hull</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>106.26798</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Man City</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Ipswich</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>106.55998</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>46312.6875</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>106.53886</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>46313.54166666666</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Bournemouth</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>106.43103</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>46313.54166666666</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Brighton</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>106.5111</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>46313.54166666666</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>106.34403</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>46313.64583333334</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Nott'm Forest</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>106.58742</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>46291.39188657407</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
         <v>46314.79166666666</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Tottenham</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Coventry</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>BetExplorer best odds</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="n">
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>BetExplorer best odds</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
         <v>1.48</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="F29" s="2" t="n">
         <v>4.48</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>5.93</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="H29" s="6" t="n">
         <v>106.7524</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I29" s="5" t="n">
         <v>46291.39188657407</v>
       </c>
     </row>
@@ -2282,24 +2605,298 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Date match</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Domicile</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Extérieur</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Ancienne cote</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Nouvelle cote</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Variation (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Date snapshot précédent</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Date snapshot actuel</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Ancienne proba (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Nouvelle proba (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Gain de proba (pts)</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Cote Fair actuelle</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Signal Marché</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Reversal Intensity (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>46292.63541666666</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Panserraikos</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Olympiacos Piraeus B</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0.2244897959183673</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>46291.4675462963</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>46291.47834490741</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.1024378809188936</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0.08373904721363497</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>-0.01869883370525861</v>
+      </c>
+      <c r="M2" s="8" t="n">
+        <v>11.94186025843835</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>TREND CONTINUATION</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>46292.63541666666</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Panserraikos</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Olympiacos Piraeus B</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0.07004830917874397</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>46291.4675462963</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>46291.47834490741</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.2182372245663385</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.2041493701822252</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>-0.01408785438411331</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>4.898374161563137</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>TREND CONTINUATION</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>46292.63541666666</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Panserraikos</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Olympiacos Piraeus B</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>-0.04511278195488721</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>46291.4675462963</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>46291.47834490741</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.679324894514768</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.7121115826041399</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0.03278668808937191</v>
+      </c>
+      <c r="M4" s="8" t="n">
+        <v>1.404274308168213</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>TREND CONTINUATION</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2:G4">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>$G2&lt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>$G2&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N4">
+    <cfRule type="expression" priority="2" dxfId="3">
+      <formula>LEFT($N2,14)="SHARP REVERSAL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2325,61 +2922,1417 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Ancienne cote</t>
+          <t>Anticipation (h)</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Nouvelle cote</t>
+          <t>Cote Prise</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Variation (%)</t>
+          <t>Cote Clôture</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Date snapshot précédent</t>
+          <t>CLV (%)</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Date snapshot actuel</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>Ancienne proba (%)</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>Nouvelle proba (%)</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
-        <is>
-          <t>Gain de proba (pts)</t>
-        </is>
-      </c>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>Cote Fair actuelle</t>
-        </is>
-      </c>
-      <c r="N1" s="3" t="inlineStr">
-        <is>
-          <t>Signal Marché</t>
-        </is>
-      </c>
-      <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>Reversal Intensity (%)</t>
+          <t>Gain Fair Proba (pts)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Date coup d'envoi UTC</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Compétition</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Équipe Domicile</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Équipe Extérieur</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Cote 1 (Ouverture)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Cote 1 (Actuelle)</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Drift 1 (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Cote 2 (Ouverture)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Cote 2 (Actuelle)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Drift 2 (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>CLV Favorable (Oui/Non)</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Nb Snapshots capturés</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>46305.47916666666</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Bournemouth</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Ipswich</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Brighton</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>46305.6875</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Tottenham</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>46306.54166666666</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Nott'm Forest</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>46306.54166666666</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Hull</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>46306.64583333334</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Man City</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>46307.79166666666</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Coventry</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>46312.47916666666</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Hull</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>46312.58333333334</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Man City</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Ipswich</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>46312.6875</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>46313.54166666666</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Bournemouth</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>46313.54166666666</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Brighton</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Crystal Palace</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>46313.54166666666</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Man United</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>46313.64583333334</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Nott'm Forest</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>46314.79166666666</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Tottenham</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Coventry</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>En attente de snapshots (T0 unique)</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>46293.54166666666</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Athens Kallithea</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Asteras Tripolis B</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>46293.54166666666</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Marko</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Panthrakikos</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>-0.01598837209302328</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>AEL Larissa</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>PAOK B</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Kalamaria</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Karditsa</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>-0.003003003003003046</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Niki Volos</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Chrisoupolis</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Panionios</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Zakynthos</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>46292.58333333334</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Ellas Syrou</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Pyrgos</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="L28" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>46292.63541666666</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Super League 2</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Panserraikos</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Olympiacos Piraeus B</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>-0.04511278195488721</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>0.2471655328798186</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="K2:K29">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>$K2="Oui"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$K2="Non"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>